<commit_message>
Change NaN to NA for N2
</commit_message>
<xml_diff>
--- a/tableS1/Table_S1.xlsx
+++ b/tableS1/Table_S1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="5137" uniqueCount="2211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="5199" uniqueCount="2251">
   <si>
     <t>Strain_Name</t>
   </si>
@@ -5710,12 +5710,6 @@
     <t>CF367</t>
   </si>
   <si>
-    <t>CFY13</t>
-  </si>
-  <si>
-    <t>CHS1198</t>
-  </si>
-  <si>
     <t>CZ26389</t>
   </si>
   <si>
@@ -5740,9 +5734,6 @@
     <t>EU640</t>
   </si>
   <si>
-    <t>FX1053</t>
-  </si>
-  <si>
     <t>FX627</t>
   </si>
   <si>
@@ -5752,9 +5743,6 @@
     <t>IG544</t>
   </si>
   <si>
-    <t>IK581</t>
-  </si>
-  <si>
     <t>IK777</t>
   </si>
   <si>
@@ -5866,9 +5854,6 @@
     <t>RB2572</t>
   </si>
   <si>
-    <t>RB2591</t>
-  </si>
-  <si>
     <t>RB684</t>
   </si>
   <si>
@@ -5899,9 +5884,6 @@
     <t>UV26</t>
   </si>
   <si>
-    <t>VC1099</t>
-  </si>
-  <si>
     <t>VC1293</t>
   </si>
   <si>
@@ -5947,15 +5929,9 @@
     <t>VC356</t>
   </si>
   <si>
-    <t>VC364</t>
-  </si>
-  <si>
     <t>VC387</t>
   </si>
   <si>
-    <t>VC475</t>
-  </si>
-  <si>
     <t>VC596</t>
   </si>
   <si>
@@ -6001,9 +5977,6 @@
     <t>tm3373</t>
   </si>
   <si>
-    <t>tm4050</t>
-  </si>
-  <si>
     <t>tm5036</t>
   </si>
   <si>
@@ -6028,12 +6001,6 @@
     <t>mig-14(mu71) II.</t>
   </si>
   <si>
-    <t>C27D6.11(syb11016) II.</t>
-  </si>
-  <si>
-    <t>srv-1(yum2185) srv-2(yum2186) srv-3(yum2187) srv-4(yum2188) srv-17(yum2189) srv-19(yum2190) srv-21(yum2191) srv-22(yum2192) srv-34(yum2193) III.</t>
-  </si>
-  <si>
     <t>esyt-2(ju1408) III.</t>
   </si>
   <si>
@@ -6058,9 +6025,6 @@
     <t>cul-2(or209) III.</t>
   </si>
   <si>
-    <t>ins-11(tm1053) II.</t>
-  </si>
-  <si>
     <t>lgc-11(tm627) X.</t>
   </si>
   <si>
@@ -6070,9 +6034,6 @@
     <t>nipi-3(fr4) X.</t>
   </si>
   <si>
-    <t>ins-1(nj32) IV.</t>
-  </si>
-  <si>
     <t>egl-8(nj77) V. Outcrossed x5</t>
   </si>
   <si>
@@ -6184,9 +6145,6 @@
     <t>Y38F1A.6(ok3580) II.</t>
   </si>
   <si>
-    <t>C27D6.11(ok3612) II.</t>
-  </si>
-  <si>
     <t>tank-1(ok446) V.</t>
   </si>
   <si>
@@ -6217,9 +6175,6 @@
     <t>him-19(tm3538) I.</t>
   </si>
   <si>
-    <t>hsp-4(gk514) II.</t>
-  </si>
-  <si>
     <t>F45C12.3(gk583) II.</t>
   </si>
   <si>
@@ -6265,15 +6220,9 @@
     <t>tag-77(gk206) IV.</t>
   </si>
   <si>
-    <t>tbb-1(gk207) III.</t>
-  </si>
-  <si>
     <t>cla-1(ok618) IV.</t>
   </si>
   <si>
-    <t>hsp-16.2(gk249) V.</t>
-  </si>
-  <si>
     <t>cla-1(gk352) IV.</t>
   </si>
   <si>
@@ -6319,9 +6268,6 @@
     <t>K09A9.1/tmC24(tm3373) X.</t>
   </si>
   <si>
-    <t>C27D6.11(tm4050) II.</t>
-  </si>
-  <si>
     <t>che-6(tm5036) IV.</t>
   </si>
   <si>
@@ -6346,12 +6292,6 @@
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00004822#03--10</t>
   </si>
   <si>
-    <t>Fang-Yen Lab Strain Collection: CFY13</t>
-  </si>
-  <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00062447#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00049860#03--10</t>
   </si>
   <si>
@@ -6376,9 +6316,6 @@
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00007297#03--10</t>
   </si>
   <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00007572#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00007565#03--10</t>
   </si>
   <si>
@@ -6388,9 +6325,6 @@
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00021982#03--10</t>
   </si>
   <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00022000#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00022014#03--10</t>
   </si>
   <si>
@@ -6502,9 +6436,6 @@
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00033247#03--10</t>
   </si>
   <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00033266#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00031422#03--10</t>
   </si>
   <si>
@@ -6535,9 +6466,6 @@
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00035462#03--10</t>
   </si>
   <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00036323#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00036486#03--10</t>
   </si>
   <si>
@@ -6583,15 +6511,9 @@
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00035705#03--10</t>
   </si>
   <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00035711#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00035728#03--10</t>
   </si>
   <si>
-    <t>https://wormbase.org/species/c_elegans/strain/WBStrain00035801#03--10</t>
-  </si>
-  <si>
     <t>https://wormbase.org/species/c_elegans/strain/WBStrain00035905#03--10</t>
   </si>
   <si>
@@ -6637,16 +6559,214 @@
     <t>https://shigen.nig.ac.jp/c.elegans/DetailsSearch?allele=tm3373</t>
   </si>
   <si>
-    <t>https://shigen.nig.ac.jp/c.elegans/DetailsSearch?allele=tm4050</t>
-  </si>
-  <si>
     <t>https://shigen.nig.ac.jp/c.elegans/DetailsSearch?allele=tm5036</t>
   </si>
   <si>
-    <t>Fang-Yen Lab</t>
-  </si>
-  <si>
     <t>National BioResource Project (Japan)</t>
+  </si>
+  <si>
+    <t>SKAT_Rank_Percentile</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>7.29</t>
+  </si>
+  <si>
+    <t>1.49</t>
+  </si>
+  <si>
+    <t>0.45</t>
+  </si>
+  <si>
+    <t>0.23</t>
+  </si>
+  <si>
+    <t>12.37</t>
+  </si>
+  <si>
+    <t>1.73</t>
+  </si>
+  <si>
+    <t>12.88</t>
+  </si>
+  <si>
+    <t>2.7</t>
+  </si>
+  <si>
+    <t>0.36</t>
+  </si>
+  <si>
+    <t>2.04</t>
+  </si>
+  <si>
+    <t>0.68</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>7.5</t>
+  </si>
+  <si>
+    <t>13.45</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>1.34</t>
+  </si>
+  <si>
+    <t>6.15</t>
+  </si>
+  <si>
+    <t>12.92</t>
+  </si>
+  <si>
+    <t>0.93</t>
+  </si>
+  <si>
+    <t>1.31</t>
+  </si>
+  <si>
+    <t>0.24</t>
+  </si>
+  <si>
+    <t>3.21</t>
+  </si>
+  <si>
+    <t>0.14</t>
+  </si>
+  <si>
+    <t>2.81</t>
+  </si>
+  <si>
+    <t>10.51</t>
+  </si>
+  <si>
+    <t>0.75</t>
+  </si>
+  <si>
+    <t>20.17</t>
+  </si>
+  <si>
+    <t>8.06</t>
+  </si>
+  <si>
+    <t>0.27</t>
+  </si>
+  <si>
+    <t>12.32</t>
+  </si>
+  <si>
+    <t>12.91</t>
+  </si>
+  <si>
+    <t>49.51</t>
+  </si>
+  <si>
+    <t>1.41</t>
+  </si>
+  <si>
+    <t>0.05</t>
+  </si>
+  <si>
+    <t>1.04</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>5.51</t>
+  </si>
+  <si>
+    <t>0.71</t>
+  </si>
+  <si>
+    <t>1.35</t>
+  </si>
+  <si>
+    <t>0.02</t>
+  </si>
+  <si>
+    <t>1.68</t>
+  </si>
+  <si>
+    <t>15.29</t>
+  </si>
+  <si>
+    <t>1.17</t>
+  </si>
+  <si>
+    <t>8.7</t>
+  </si>
+  <si>
+    <t>3.02</t>
+  </si>
+  <si>
+    <t>5.45</t>
+  </si>
+  <si>
+    <t>1.13</t>
+  </si>
+  <si>
+    <t>2.33</t>
+  </si>
+  <si>
+    <t>0.47</t>
+  </si>
+  <si>
+    <t>11.33</t>
+  </si>
+  <si>
+    <t>1.79</t>
+  </si>
+  <si>
+    <t>1.28</t>
+  </si>
+  <si>
+    <t>13.42</t>
+  </si>
+  <si>
+    <t>3.3</t>
+  </si>
+  <si>
+    <t>0.42</t>
+  </si>
+  <si>
+    <t>13.27</t>
+  </si>
+  <si>
+    <t>0.18</t>
+  </si>
+  <si>
+    <t>32.97</t>
+  </si>
+  <si>
+    <t>16.91</t>
+  </si>
+  <si>
+    <t>18.39</t>
+  </si>
+  <si>
+    <t>0.08</t>
+  </si>
+  <si>
+    <t>58.04</t>
+  </si>
+  <si>
+    <t>1.55</t>
+  </si>
+  <si>
+    <t>11.8</t>
+  </si>
+  <si>
+    <t>0.99</t>
+  </si>
+  <si>
+    <t>25.53</t>
   </si>
 </sst>
 </file>
@@ -28353,15 +28473,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="true"/>
-    <col min="2" max="2" width="134.42578125" customWidth="true"/>
+    <col min="2" max="2" width="33.42578125" customWidth="true"/>
     <col min="3" max="3" width="67" customWidth="true"/>
     <col min="4" max="4" width="33.7109375" customWidth="true"/>
     <col min="5" max="5" width="26.140625" customWidth="true"/>
     <col min="6" max="6" width="27" customWidth="true"/>
+    <col min="7" max="7" width="21" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -28383,16 +28504,19 @@
       <c r="F1" s="0" t="s">
         <v>1890</v>
       </c>
+      <c r="G1" s="0" t="s">
+        <v>2183</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
         <v>1891</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>1997</v>
+        <v>1988</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>2103</v>
+        <v>2085</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>1885</v>
@@ -28402,6 +28526,9 @@
       </c>
       <c r="F2" s="0">
         <v>0.61160714285714302</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>2184</v>
       </c>
     </row>
     <row r="3">
@@ -28409,10 +28536,10 @@
         <v>1892</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>1998</v>
+        <v>1989</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>2104</v>
+        <v>2086</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>1885</v>
@@ -28422,6 +28549,9 @@
       </c>
       <c r="F3" s="0">
         <v>0.61643026004728097</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>2185</v>
       </c>
     </row>
     <row r="4">
@@ -28429,10 +28559,10 @@
         <v>1893</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>1999</v>
+        <v>1990</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>2105</v>
+        <v>2087</v>
       </c>
       <c r="D4" s="0" t="s">
         <v>1885</v>
@@ -28442,6 +28572,9 @@
       </c>
       <c r="F4" s="0">
         <v>0.61134259259259305</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>2185</v>
       </c>
     </row>
     <row r="5">
@@ -28449,10 +28582,10 @@
         <v>1894</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>2000</v>
+        <v>1991</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>2106</v>
+        <v>2088</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>1885</v>
@@ -28462,6 +28595,9 @@
       </c>
       <c r="F5" s="0">
         <v>0.67872942386831303</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>2185</v>
       </c>
     </row>
     <row r="6">
@@ -28469,10 +28605,10 @@
         <v>1895</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>2001</v>
+        <v>1992</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>2107</v>
+        <v>2089</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>1885</v>
@@ -28482,6 +28618,9 @@
       </c>
       <c r="F6" s="0">
         <v>0.68583333333333296</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>2186</v>
       </c>
     </row>
     <row r="7">
@@ -28489,10 +28628,10 @@
         <v>1896</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>2002</v>
+        <v>1993</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>2108</v>
+        <v>2090</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>1885</v>
@@ -28502,6 +28641,9 @@
       </c>
       <c r="F7" s="0">
         <v>0.79801793981481495</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>2187</v>
       </c>
     </row>
     <row r="8">
@@ -28509,10 +28651,10 @@
         <v>1897</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>2003</v>
+        <v>1994</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>2109</v>
+        <v>2091</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>1885</v>
@@ -28522,6 +28664,9 @@
       </c>
       <c r="F8" s="0">
         <v>0.57853009259259203</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>2188</v>
       </c>
     </row>
     <row r="9">
@@ -28529,19 +28674,22 @@
         <v>1898</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>2004</v>
+        <v>1995</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>2110</v>
+        <v>2092</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>2209</v>
+        <v>1885</v>
       </c>
       <c r="E9" s="0">
-        <v>0.042994966442953003</v>
+        <v>0.087248322147651006</v>
       </c>
       <c r="F9" s="0">
-        <v>0.57404513888888897</v>
+        <v>0.62092013888888897</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>2189</v>
       </c>
     </row>
     <row r="10">
@@ -28549,19 +28697,22 @@
         <v>1899</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>2005</v>
+        <v>1996</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>2111</v>
+        <v>2093</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E10" s="0">
-        <v>0.0304054054054054</v>
+        <v>0.18076645677316799</v>
       </c>
       <c r="F10" s="0">
-        <v>0.593287037037037</v>
+        <v>0.58556547619047605</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>2190</v>
       </c>
     </row>
     <row r="11">
@@ -28569,19 +28720,22 @@
         <v>1900</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>2006</v>
+        <v>1997</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>2112</v>
+        <v>2094</v>
       </c>
       <c r="D11" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E11" s="0">
-        <v>0.087248322147651006</v>
+        <v>0.14988814317673399</v>
       </c>
       <c r="F11" s="0">
-        <v>0.62092013888888897</v>
+        <v>0.70138888888888895</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>2190</v>
       </c>
     </row>
     <row r="12">
@@ -28589,19 +28743,22 @@
         <v>1901</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>2007</v>
+        <v>1998</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>2113</v>
+        <v>2095</v>
       </c>
       <c r="D12" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E12" s="0">
-        <v>0.18076645677316799</v>
+        <v>0.29773982499046098</v>
       </c>
       <c r="F12" s="0">
-        <v>0.58556547619047605</v>
+        <v>0.64578544061302701</v>
+      </c>
+      <c r="G12" s="0" t="s">
+        <v>2190</v>
       </c>
     </row>
     <row r="13">
@@ -28609,19 +28766,22 @@
         <v>1902</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>2008</v>
+        <v>1999</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>2114</v>
+        <v>2096</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E13" s="0">
-        <v>0.14988814317673399</v>
+        <v>0.14643075045759599</v>
       </c>
       <c r="F13" s="0">
-        <v>0.70138888888888895</v>
+        <v>0.61388888888888904</v>
+      </c>
+      <c r="G13" s="0" t="s">
+        <v>2190</v>
       </c>
     </row>
     <row r="14">
@@ -28629,19 +28789,22 @@
         <v>1903</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>2009</v>
+        <v>2000</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>2115</v>
+        <v>2097</v>
       </c>
       <c r="D14" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E14" s="0">
-        <v>0.29773982499046098</v>
+        <v>0</v>
       </c>
       <c r="F14" s="0">
-        <v>0.64578544061302701</v>
+        <v>0.567512077294686</v>
+      </c>
+      <c r="G14" s="0" t="s">
+        <v>2191</v>
       </c>
     </row>
     <row r="15">
@@ -28649,19 +28812,22 @@
         <v>1904</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>2010</v>
+        <v>2001</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>2116</v>
+        <v>2098</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E15" s="0">
-        <v>0.14643075045759599</v>
+        <v>0.057432432432432401</v>
       </c>
       <c r="F15" s="0">
-        <v>0.61388888888888904</v>
+        <v>0.53869047619047605</v>
+      </c>
+      <c r="G15" s="0" t="s">
+        <v>2192</v>
       </c>
     </row>
     <row r="16">
@@ -28669,19 +28835,22 @@
         <v>1905</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>2011</v>
+        <v>2002</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>2117</v>
+        <v>2099</v>
       </c>
       <c r="D16" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E16" s="0">
-        <v>0</v>
+        <v>0.10022522522522501</v>
       </c>
       <c r="F16" s="0">
-        <v>0.567512077294686</v>
+        <v>0.62787037037036997</v>
+      </c>
+      <c r="G16" s="0" t="s">
+        <v>2193</v>
       </c>
     </row>
     <row r="17">
@@ -28689,19 +28858,22 @@
         <v>1906</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>2012</v>
+        <v>2003</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>2118</v>
+        <v>2100</v>
       </c>
       <c r="D17" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E17" s="0">
-        <v>0.057432432432432401</v>
+        <v>0.060360360360360403</v>
       </c>
       <c r="F17" s="0">
-        <v>0.53869047619047605</v>
+        <v>0.62439814814814798</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>2194</v>
       </c>
     </row>
     <row r="18">
@@ -28709,19 +28881,22 @@
         <v>1907</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>2013</v>
+        <v>2004</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>2119</v>
+        <v>2101</v>
       </c>
       <c r="D18" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E18" s="0">
-        <v>0.10022522522522501</v>
+        <v>0.032818532818532802</v>
       </c>
       <c r="F18" s="0">
-        <v>0.62787037037036997</v>
+        <v>0.60342261904761896</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>2195</v>
       </c>
     </row>
     <row r="19">
@@ -28729,19 +28904,22 @@
         <v>1908</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>2014</v>
+        <v>2005</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>2120</v>
+        <v>2102</v>
       </c>
       <c r="D19" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E19" s="0">
-        <v>0.109619686800895</v>
+        <v>0.13327120223671901</v>
       </c>
       <c r="F19" s="0">
-        <v>0.59972222222222205</v>
+        <v>0.65711206896551699</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>2196</v>
       </c>
     </row>
     <row r="20">
@@ -28749,19 +28927,22 @@
         <v>1909</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>2015</v>
+        <v>2006</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>2121</v>
+        <v>2103</v>
       </c>
       <c r="D20" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E20" s="0">
-        <v>0.060360360360360403</v>
+        <v>0.075090841003376194</v>
       </c>
       <c r="F20" s="0">
-        <v>0.62439814814814798</v>
+        <v>0.77896505376344105</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>2187</v>
       </c>
     </row>
     <row r="21">
@@ -28769,19 +28950,22 @@
         <v>1910</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>2016</v>
+        <v>2007</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>2122</v>
+        <v>2104</v>
       </c>
       <c r="D21" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E21" s="0">
-        <v>0.032818532818532802</v>
+        <v>0.072840371035233303</v>
       </c>
       <c r="F21" s="0">
-        <v>0.60342261904761896</v>
+        <v>0.88975095785440605</v>
+      </c>
+      <c r="G21" s="0" t="s">
+        <v>2187</v>
       </c>
     </row>
     <row r="22">
@@ -28789,19 +28973,22 @@
         <v>1911</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>2017</v>
+        <v>2008</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>2123</v>
+        <v>2105</v>
       </c>
       <c r="D22" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E22" s="0">
-        <v>0.13327120223671901</v>
+        <v>0.20134228187919501</v>
       </c>
       <c r="F22" s="0">
-        <v>0.65711206896551699</v>
+        <v>0.65905349794238699</v>
+      </c>
+      <c r="G22" s="0" t="s">
+        <v>2197</v>
       </c>
     </row>
     <row r="23">
@@ -28809,19 +28996,22 @@
         <v>1912</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>2018</v>
+        <v>2009</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>2124</v>
+        <v>2106</v>
       </c>
       <c r="D23" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E23" s="0">
-        <v>0.078096400244051206</v>
+        <v>0.062952213958925404</v>
       </c>
       <c r="F23" s="0">
-        <v>0.55077861952861995</v>
+        <v>0.92752057613168704</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>2187</v>
       </c>
     </row>
     <row r="24">
@@ -28829,19 +29019,22 @@
         <v>1913</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>2019</v>
+        <v>2010</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>2125</v>
+        <v>2107</v>
       </c>
       <c r="D24" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E24" s="0">
-        <v>0.075090841003376194</v>
+        <v>0.0352348993288591</v>
       </c>
       <c r="F24" s="0">
-        <v>0.77896505376344105</v>
+        <v>0.60251736111111098</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>2198</v>
       </c>
     </row>
     <row r="25">
@@ -28849,19 +29042,22 @@
         <v>1914</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>2020</v>
+        <v>2011</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>2126</v>
+        <v>2108</v>
       </c>
       <c r="D25" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E25" s="0">
-        <v>0.072840371035233303</v>
+        <v>0.073768048039351303</v>
       </c>
       <c r="F25" s="0">
-        <v>0.88975095785440605</v>
+        <v>0.58468956270627104</v>
+      </c>
+      <c r="G25" s="0" t="s">
+        <v>2199</v>
       </c>
     </row>
     <row r="26">
@@ -28869,19 +29065,22 @@
         <v>1915</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>2127</v>
+        <v>2109</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E26" s="0">
-        <v>0.20134228187919501</v>
+        <v>0.00213544844417328</v>
       </c>
       <c r="F26" s="0">
-        <v>0.65905349794238699</v>
+        <v>0.54797979797979801</v>
+      </c>
+      <c r="G26" s="0" t="s">
+        <v>2200</v>
       </c>
     </row>
     <row r="27">
@@ -28889,19 +29088,22 @@
         <v>1916</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>2022</v>
+        <v>2013</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>2128</v>
+        <v>2110</v>
       </c>
       <c r="D27" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E27" s="0">
-        <v>0.062952213958925404</v>
+        <v>0.160544217687075</v>
       </c>
       <c r="F27" s="0">
-        <v>0.92752057613168704</v>
+        <v>0.59212962962963001</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>2201</v>
       </c>
     </row>
     <row r="28">
@@ -28909,19 +29111,22 @@
         <v>1917</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>2023</v>
+        <v>2014</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>2129</v>
+        <v>2111</v>
       </c>
       <c r="D28" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E28" s="0">
-        <v>0.0352348993288591</v>
+        <v>0.0276446893549416</v>
       </c>
       <c r="F28" s="0">
-        <v>0.60251736111111098</v>
+        <v>0.63359674329501903</v>
+      </c>
+      <c r="G28" s="0" t="s">
+        <v>2202</v>
       </c>
     </row>
     <row r="29">
@@ -28929,19 +29134,22 @@
         <v>1918</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>2024</v>
+        <v>2015</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>2130</v>
+        <v>2112</v>
       </c>
       <c r="D29" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E29" s="0">
-        <v>0.073768048039351303</v>
+        <v>0.044378438841526098</v>
       </c>
       <c r="F29" s="0">
-        <v>0.58468956270627104</v>
+        <v>0.55594907407407401</v>
+      </c>
+      <c r="G29" s="0" t="s">
+        <v>2202</v>
       </c>
     </row>
     <row r="30">
@@ -28949,19 +29157,22 @@
         <v>1919</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>2025</v>
+        <v>2016</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>2131</v>
+        <v>2113</v>
       </c>
       <c r="D30" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E30" s="0">
-        <v>0.00213544844417328</v>
+        <v>0.062741312741312699</v>
       </c>
       <c r="F30" s="0">
-        <v>0.54797979797979801</v>
+        <v>0.54861111111111105</v>
+      </c>
+      <c r="G30" s="0" t="s">
+        <v>2203</v>
       </c>
     </row>
     <row r="31">
@@ -28969,19 +29180,22 @@
         <v>1920</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>2026</v>
+        <v>2017</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>2132</v>
+        <v>2114</v>
       </c>
       <c r="D31" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E31" s="0">
-        <v>0.160544217687075</v>
+        <v>0.029362416107382501</v>
       </c>
       <c r="F31" s="0">
-        <v>0.59212962962963001</v>
+        <v>0.56245659722222197</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>2204</v>
       </c>
     </row>
     <row r="32">
@@ -28989,19 +29203,22 @@
         <v>1921</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>2027</v>
+        <v>2018</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>2133</v>
+        <v>2115</v>
       </c>
       <c r="D32" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E32" s="0">
-        <v>0.0276446893549416</v>
+        <v>0.136744966442953</v>
       </c>
       <c r="F32" s="0">
-        <v>0.63359674329501903</v>
+        <v>0.58849826388888904</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>2205</v>
       </c>
     </row>
     <row r="33">
@@ -29009,19 +29226,22 @@
         <v>1922</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>2028</v>
+        <v>2019</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>2134</v>
+        <v>2116</v>
       </c>
       <c r="D33" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E33" s="0">
-        <v>0.044378438841526098</v>
+        <v>0.057885906040268401</v>
       </c>
       <c r="F33" s="0">
-        <v>0.55594907407407401</v>
+        <v>0.59247685185185195</v>
+      </c>
+      <c r="G33" s="0" t="s">
+        <v>2206</v>
       </c>
     </row>
     <row r="34">
@@ -29029,19 +29249,22 @@
         <v>1923</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>2029</v>
+        <v>2020</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>2135</v>
+        <v>2117</v>
       </c>
       <c r="D34" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E34" s="0">
-        <v>0.062741312741312699</v>
+        <v>0.105076313130004</v>
       </c>
       <c r="F34" s="0">
-        <v>0.54861111111111105</v>
+        <v>0.51441468253968203</v>
+      </c>
+      <c r="G34" s="0" t="s">
+        <v>2207</v>
       </c>
     </row>
     <row r="35">
@@ -29049,19 +29272,22 @@
         <v>1924</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>2030</v>
+        <v>2021</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>2136</v>
+        <v>2118</v>
       </c>
       <c r="D35" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E35" s="0">
-        <v>0.029362416107382501</v>
+        <v>0.0071308724832214801</v>
       </c>
       <c r="F35" s="0">
-        <v>0.56245659722222197</v>
+        <v>0.60546875</v>
+      </c>
+      <c r="G35" s="0" t="s">
+        <v>2200</v>
       </c>
     </row>
     <row r="36">
@@ -29069,19 +29295,22 @@
         <v>1925</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>2031</v>
+        <v>2022</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>2137</v>
+        <v>2119</v>
       </c>
       <c r="D36" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E36" s="0">
-        <v>0.136744966442953</v>
+        <v>0.13963963963963999</v>
       </c>
       <c r="F36" s="0">
-        <v>0.58849826388888904</v>
+        <v>0.66273148148148098</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>2208</v>
       </c>
     </row>
     <row r="37">
@@ -29089,19 +29318,22 @@
         <v>1926</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>2032</v>
+        <v>2023</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>2138</v>
+        <v>2120</v>
       </c>
       <c r="D37" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E37" s="0">
-        <v>0.057885906040268401</v>
+        <v>0.077922077922077906</v>
       </c>
       <c r="F37" s="0">
-        <v>0.59247685185185195</v>
+        <v>0.60843253968253996</v>
+      </c>
+      <c r="G37" s="0" t="s">
+        <v>2209</v>
       </c>
     </row>
     <row r="38">
@@ -29109,19 +29341,22 @@
         <v>1927</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>2033</v>
+        <v>2024</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>2139</v>
+        <v>2121</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E38" s="0">
-        <v>0.105076313130004</v>
+        <v>0.21349820877924899</v>
       </c>
       <c r="F38" s="0">
-        <v>0.51441468253968203</v>
+        <v>0.61486545138888904</v>
+      </c>
+      <c r="G38" s="0" t="s">
+        <v>2210</v>
       </c>
     </row>
     <row r="39">
@@ -29129,19 +29364,22 @@
         <v>1928</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>2034</v>
+        <v>2025</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>2140</v>
+        <v>2122</v>
       </c>
       <c r="D39" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E39" s="0">
-        <v>0.0071308724832214801</v>
+        <v>0.0103305785123967</v>
       </c>
       <c r="F39" s="0">
-        <v>0.60546875</v>
+        <v>0.63103298611111103</v>
+      </c>
+      <c r="G39" s="0" t="s">
+        <v>2211</v>
       </c>
     </row>
     <row r="40">
@@ -29149,19 +29387,22 @@
         <v>1929</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>2035</v>
+        <v>2026</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>2141</v>
+        <v>2123</v>
       </c>
       <c r="D40" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E40" s="0">
-        <v>0.13963963963963999</v>
+        <v>0.051691197462063597</v>
       </c>
       <c r="F40" s="0">
-        <v>0.66273148148148098</v>
+        <v>0.50464559386973196</v>
+      </c>
+      <c r="G40" s="0" t="s">
+        <v>2212</v>
       </c>
     </row>
     <row r="41">
@@ -29169,19 +29410,22 @@
         <v>1930</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>2036</v>
+        <v>2027</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>2142</v>
+        <v>2124</v>
       </c>
       <c r="D41" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E41" s="0">
-        <v>0.077922077922077906</v>
+        <v>0.18597668668315101</v>
       </c>
       <c r="F41" s="0">
-        <v>0.60843253968253996</v>
+        <v>0.72898391812865504</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>2213</v>
       </c>
     </row>
     <row r="42">
@@ -29189,19 +29433,22 @@
         <v>1931</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>2037</v>
+        <v>2028</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>2143</v>
+        <v>2125</v>
       </c>
       <c r="D42" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E42" s="0">
-        <v>0.21349820877924899</v>
+        <v>0.23463745229635499</v>
       </c>
       <c r="F42" s="0">
-        <v>0.61486545138888904</v>
+        <v>0.51542592592592595</v>
+      </c>
+      <c r="G42" s="0" t="s">
+        <v>2214</v>
       </c>
     </row>
     <row r="43">
@@ -29209,19 +29456,22 @@
         <v>1932</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>2038</v>
+        <v>2029</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>2144</v>
+        <v>2126</v>
       </c>
       <c r="D43" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E43" s="0">
-        <v>0.0103305785123967</v>
+        <v>0.18603423572882899</v>
       </c>
       <c r="F43" s="0">
-        <v>0.63103298611111103</v>
+        <v>0.396410736579276</v>
+      </c>
+      <c r="G43" s="0" t="s">
+        <v>2215</v>
       </c>
     </row>
     <row r="44">
@@ -29229,19 +29479,22 @@
         <v>1933</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>2039</v>
+        <v>2030</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>2145</v>
+        <v>2127</v>
       </c>
       <c r="D44" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E44" s="0">
-        <v>0.051691197462063597</v>
+        <v>0.042684497497405501</v>
       </c>
       <c r="F44" s="0">
-        <v>0.50464559386973196</v>
+        <v>0.499537037037037</v>
+      </c>
+      <c r="G44" s="0" t="s">
+        <v>2215</v>
       </c>
     </row>
     <row r="45">
@@ -29249,19 +29502,22 @@
         <v>1934</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>2040</v>
+        <v>2031</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>2146</v>
+        <v>2128</v>
       </c>
       <c r="D45" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E45" s="0">
-        <v>0.18597668668315101</v>
+        <v>0.151492742096769</v>
       </c>
       <c r="F45" s="0">
-        <v>0.72898391812865504</v>
+        <v>0.70849358974359</v>
+      </c>
+      <c r="G45" s="0" t="s">
+        <v>2216</v>
       </c>
     </row>
     <row r="46">
@@ -29269,19 +29525,22 @@
         <v>1935</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>2041</v>
+        <v>2032</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>2147</v>
+        <v>2129</v>
       </c>
       <c r="D46" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E46" s="0">
-        <v>0.23463745229635499</v>
+        <v>0.025337837837837801</v>
       </c>
       <c r="F46" s="0">
-        <v>0.51542592592592595</v>
+        <v>0.55264756944444404</v>
+      </c>
+      <c r="G46" s="0" t="s">
+        <v>2217</v>
       </c>
     </row>
     <row r="47">
@@ -29289,19 +29548,22 @@
         <v>1936</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>2042</v>
+        <v>2033</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>2148</v>
+        <v>2130</v>
       </c>
       <c r="D47" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E47" s="0">
-        <v>0.18603423572882899</v>
+        <v>0.049876121758848702</v>
       </c>
       <c r="F47" s="0">
-        <v>0.396410736579276</v>
+        <v>0.678015350877193</v>
+      </c>
+      <c r="G47" s="0" t="s">
+        <v>2218</v>
       </c>
     </row>
     <row r="48">
@@ -29309,19 +29571,22 @@
         <v>1937</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>2043</v>
+        <v>2034</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>2149</v>
+        <v>2131</v>
       </c>
       <c r="D48" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E48" s="0">
-        <v>0.042684497497405501</v>
+        <v>0.057432432432432401</v>
       </c>
       <c r="F48" s="0">
-        <v>0.499537037037037</v>
+        <v>0.61850198412698398</v>
+      </c>
+      <c r="G48" s="0" t="s">
+        <v>2219</v>
       </c>
     </row>
     <row r="49">
@@ -29329,19 +29594,22 @@
         <v>1938</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>2044</v>
+        <v>2035</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>2150</v>
+        <v>2132</v>
       </c>
       <c r="D49" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E49" s="0">
-        <v>0.151492742096769</v>
+        <v>0.072782514057681796</v>
       </c>
       <c r="F49" s="0">
-        <v>0.70849358974359</v>
+        <v>0.67514367816091903</v>
+      </c>
+      <c r="G49" s="0" t="s">
+        <v>2220</v>
       </c>
     </row>
     <row r="50">
@@ -29349,19 +29617,22 @@
         <v>1939</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>2045</v>
+        <v>2036</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>2151</v>
+        <v>2133</v>
       </c>
       <c r="D50" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E50" s="0">
-        <v>0.025337837837837801</v>
+        <v>0.094439117929050798</v>
       </c>
       <c r="F50" s="0">
-        <v>0.55264756944444404</v>
+        <v>0.61160714285714302</v>
+      </c>
+      <c r="G50" s="0" t="s">
+        <v>2221</v>
       </c>
     </row>
     <row r="51">
@@ -29369,19 +29640,22 @@
         <v>1940</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>2046</v>
+        <v>2037</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>2152</v>
+        <v>2134</v>
       </c>
       <c r="D51" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E51" s="0">
-        <v>0.049876121758848702</v>
+        <v>0.31027361899845102</v>
       </c>
       <c r="F51" s="0">
-        <v>0.678015350877193</v>
+        <v>0.72008547008546997</v>
+      </c>
+      <c r="G51" s="0" t="s">
+        <v>2222</v>
       </c>
     </row>
     <row r="52">
@@ -29389,19 +29663,22 @@
         <v>1941</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>2047</v>
+        <v>2038</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>2153</v>
+        <v>2135</v>
       </c>
       <c r="D52" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E52" s="0">
-        <v>0.057432432432432401</v>
+        <v>0.22719363658961001</v>
       </c>
       <c r="F52" s="0">
-        <v>0.61850198412698398</v>
+        <v>0.577199074074074</v>
+      </c>
+      <c r="G52" s="0" t="s">
+        <v>2223</v>
       </c>
     </row>
     <row r="53">
@@ -29409,19 +29686,22 @@
         <v>1942</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>2048</v>
+        <v>2039</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>2154</v>
+        <v>2136</v>
       </c>
       <c r="D53" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E53" s="0">
-        <v>0.072782514057681796</v>
+        <v>0.073597997952451394</v>
       </c>
       <c r="F53" s="0">
-        <v>0.67514367816091903</v>
+        <v>0.43624058380414299</v>
+      </c>
+      <c r="G53" s="0" t="s">
+        <v>2224</v>
       </c>
     </row>
     <row r="54">
@@ -29429,19 +29709,22 @@
         <v>1943</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>2049</v>
+        <v>2040</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>2155</v>
+        <v>2137</v>
       </c>
       <c r="D54" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E54" s="0">
-        <v>0.094439117929050798</v>
+        <v>0.12751677852349</v>
       </c>
       <c r="F54" s="0">
-        <v>0.61160714285714302</v>
+        <v>0.55805555555555597</v>
+      </c>
+      <c r="G54" s="0" t="s">
+        <v>2225</v>
       </c>
     </row>
     <row r="55">
@@ -29449,19 +29732,22 @@
         <v>1944</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>2050</v>
+        <v>2041</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>2156</v>
+        <v>2138</v>
       </c>
       <c r="D55" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E55" s="0">
-        <v>0.31027361899845102</v>
+        <v>0.22424242424242399</v>
       </c>
       <c r="F55" s="0">
-        <v>0.72008547008546997</v>
+        <v>0.75384259259259301</v>
+      </c>
+      <c r="G55" s="0" t="s">
+        <v>2226</v>
       </c>
     </row>
     <row r="56">
@@ -29469,19 +29755,22 @@
         <v>1945</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>2051</v>
+        <v>2042</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>2157</v>
+        <v>2139</v>
       </c>
       <c r="D56" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E56" s="0">
-        <v>0.22719363658961001</v>
+        <v>0.077192038730500304</v>
       </c>
       <c r="F56" s="0">
-        <v>0.577199074074074</v>
+        <v>0.58253205128205099</v>
+      </c>
+      <c r="G56" s="0" t="s">
+        <v>2227</v>
       </c>
     </row>
     <row r="57">
@@ -29489,19 +29778,22 @@
         <v>1946</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>2052</v>
+        <v>2043</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>2158</v>
+        <v>2140</v>
       </c>
       <c r="D57" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E57" s="0">
-        <v>0.073597997952451394</v>
+        <v>0.29922779922779902</v>
       </c>
       <c r="F57" s="0">
-        <v>0.43624058380414299</v>
+        <v>0.64717261904761903</v>
+      </c>
+      <c r="G57" s="0" t="s">
+        <v>2228</v>
       </c>
     </row>
     <row r="58">
@@ -29509,19 +29801,22 @@
         <v>1947</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>2053</v>
+        <v>2044</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>2159</v>
+        <v>2141</v>
       </c>
       <c r="D58" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E58" s="0">
-        <v>0.12751677852349</v>
+        <v>0.051174496644295298</v>
       </c>
       <c r="F58" s="0">
-        <v>0.55805555555555597</v>
+        <v>0.55533854166666696</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>2229</v>
       </c>
     </row>
     <row r="59">
@@ -29529,19 +29824,22 @@
         <v>1948</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>2054</v>
+        <v>2045</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>2160</v>
+        <v>2142</v>
       </c>
       <c r="D59" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E59" s="0">
-        <v>0.22424242424242399</v>
+        <v>0.073620664345578998</v>
       </c>
       <c r="F59" s="0">
-        <v>0.75384259259259301</v>
+        <v>0.692236733001658</v>
+      </c>
+      <c r="G59" s="0" t="s">
+        <v>2216</v>
       </c>
     </row>
     <row r="60">
@@ -29549,19 +29847,22 @@
         <v>1949</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>2055</v>
+        <v>2046</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>2161</v>
+        <v>2143</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E60" s="0">
-        <v>0.077192038730500304</v>
+        <v>0.058612975391498901</v>
       </c>
       <c r="F60" s="0">
-        <v>0.58253205128205099</v>
+        <v>0.57291666666666696</v>
+      </c>
+      <c r="G60" s="0" t="s">
+        <v>2230</v>
       </c>
     </row>
     <row r="61">
@@ -29569,19 +29870,22 @@
         <v>1950</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>2056</v>
+        <v>2047</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>2162</v>
+        <v>2144</v>
       </c>
       <c r="D61" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E61" s="0">
-        <v>0.087959443934368206</v>
+        <v>0.070245292051871397</v>
       </c>
       <c r="F61" s="0">
-        <v>0.40405465949820801</v>
+        <v>0.69081284153005496</v>
+      </c>
+      <c r="G61" s="0" t="s">
+        <v>2185</v>
       </c>
     </row>
     <row r="62">
@@ -29589,19 +29893,22 @@
         <v>1951</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>2057</v>
+        <v>2048</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>2163</v>
+        <v>2145</v>
       </c>
       <c r="D62" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E62" s="0">
-        <v>0.29922779922779902</v>
+        <v>0.052013422818791899</v>
       </c>
       <c r="F62" s="0">
-        <v>0.64717261904761903</v>
+        <v>0.571571180555555</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>2231</v>
       </c>
     </row>
     <row r="63">
@@ -29609,19 +29916,22 @@
         <v>1952</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>2058</v>
+        <v>2049</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>2164</v>
+        <v>2146</v>
       </c>
       <c r="D63" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E63" s="0">
-        <v>0.051174496644295298</v>
+        <v>0.0849194832416309</v>
       </c>
       <c r="F63" s="0">
-        <v>0.55533854166666696</v>
+        <v>0.85532407407407396</v>
+      </c>
+      <c r="G63" s="0" t="s">
+        <v>2187</v>
       </c>
     </row>
     <row r="64">
@@ -29629,19 +29939,22 @@
         <v>1953</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>2059</v>
+        <v>2050</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>2165</v>
+        <v>2147</v>
       </c>
       <c r="D64" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E64" s="0">
-        <v>0.073620664345578998</v>
+        <v>0.026006711409396002</v>
       </c>
       <c r="F64" s="0">
-        <v>0.692236733001658</v>
+        <v>0.55698784722222206</v>
+      </c>
+      <c r="G64" s="0" t="s">
+        <v>2232</v>
       </c>
     </row>
     <row r="65">
@@ -29649,19 +29962,22 @@
         <v>1954</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>2060</v>
+        <v>2051</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>2166</v>
+        <v>2148</v>
       </c>
       <c r="D65" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E65" s="0">
-        <v>0.058612975391498901</v>
+        <v>0.055656934306569303</v>
       </c>
       <c r="F65" s="0">
-        <v>0.57291666666666696</v>
+        <v>0.61388888888888904</v>
+      </c>
+      <c r="G65" s="0" t="s">
+        <v>2233</v>
       </c>
     </row>
     <row r="66">
@@ -29669,19 +29985,22 @@
         <v>1955</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>2061</v>
+        <v>2052</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>2167</v>
+        <v>2149</v>
       </c>
       <c r="D66" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E66" s="0">
-        <v>0.070245292051871397</v>
+        <v>0.032138160057868098</v>
       </c>
       <c r="F66" s="0">
-        <v>0.69081284153005496</v>
+        <v>0.61296296296296304</v>
+      </c>
+      <c r="G66" s="0" t="s">
+        <v>2233</v>
       </c>
     </row>
     <row r="67">
@@ -29689,19 +30008,22 @@
         <v>1956</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>2062</v>
+        <v>2053</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>2168</v>
+        <v>2150</v>
       </c>
       <c r="D67" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E67" s="0">
-        <v>0.052013422818791899</v>
+        <v>0.045229063320688698</v>
       </c>
       <c r="F67" s="0">
-        <v>0.571571180555555</v>
+        <v>0.568900966183575</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>2234</v>
       </c>
     </row>
     <row r="68">
@@ -29709,19 +30031,22 @@
         <v>1957</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>2063</v>
+        <v>2054</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>2169</v>
+        <v>2151</v>
       </c>
       <c r="D68" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E68" s="0">
-        <v>0.0849194832416309</v>
+        <v>0.065645973154362394</v>
       </c>
       <c r="F68" s="0">
-        <v>0.85532407407407396</v>
+        <v>0.64055989583333295</v>
+      </c>
+      <c r="G68" s="0" t="s">
+        <v>2235</v>
       </c>
     </row>
     <row r="69">
@@ -29729,19 +30054,22 @@
         <v>1958</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>2064</v>
+        <v>2055</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>2170</v>
+        <v>2152</v>
       </c>
       <c r="D69" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E69" s="0">
-        <v>0.026006711409396002</v>
+        <v>0.122302293948888</v>
       </c>
       <c r="F69" s="0">
-        <v>0.55698784722222206</v>
+        <v>0.63376068376068395</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>2236</v>
       </c>
     </row>
     <row r="70">
@@ -29749,19 +30077,22 @@
         <v>1959</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>2065</v>
+        <v>2056</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>2171</v>
+        <v>2153</v>
       </c>
       <c r="D70" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E70" s="0">
-        <v>0.055656934306569303</v>
+        <v>0.067405894368252103</v>
       </c>
       <c r="F70" s="0">
-        <v>0.61388888888888904</v>
+        <v>0.57693236714975804</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>2237</v>
       </c>
     </row>
     <row r="71">
@@ -29769,19 +30100,22 @@
         <v>1960</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>2066</v>
+        <v>2057</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>2172</v>
+        <v>2154</v>
       </c>
       <c r="D71" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E71" s="0">
-        <v>0.032138160057868098</v>
+        <v>0.088422818791946301</v>
       </c>
       <c r="F71" s="0">
-        <v>0.61296296296296304</v>
+        <v>0.59718749999999998</v>
+      </c>
+      <c r="G71" s="0" t="s">
+        <v>2189</v>
       </c>
     </row>
     <row r="72">
@@ -29789,19 +30123,22 @@
         <v>1961</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>2067</v>
+        <v>2058</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>2173</v>
+        <v>2155</v>
       </c>
       <c r="D72" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E72" s="0">
-        <v>0.159043659043659</v>
+        <v>0.047717126089068099</v>
       </c>
       <c r="F72" s="0">
-        <v>0.64059829059828999</v>
+        <v>0.50627240143369201</v>
+      </c>
+      <c r="G72" s="0" t="s">
+        <v>2202</v>
       </c>
     </row>
     <row r="73">
@@ -29809,19 +30146,22 @@
         <v>1962</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>2068</v>
+        <v>2059</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>2174</v>
+        <v>2156</v>
       </c>
       <c r="D73" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E73" s="0">
-        <v>0.045229063320688698</v>
+        <v>0.049268018018018001</v>
       </c>
       <c r="F73" s="0">
-        <v>0.568900966183575</v>
+        <v>0.60853587962962896</v>
+      </c>
+      <c r="G73" s="0" t="s">
+        <v>2238</v>
       </c>
     </row>
     <row r="74">
@@ -29829,19 +30169,22 @@
         <v>1963</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>2069</v>
+        <v>2060</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>2175</v>
+        <v>2157</v>
       </c>
       <c r="D74" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E74" s="0">
-        <v>0.065645973154362394</v>
+        <v>0.056385739846252898</v>
       </c>
       <c r="F74" s="0">
-        <v>0.64055989583333295</v>
+        <v>0.66456552706552696</v>
+      </c>
+      <c r="G74" s="0" t="s">
+        <v>2238</v>
       </c>
     </row>
     <row r="75">
@@ -29849,19 +30192,22 @@
         <v>1964</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>2070</v>
+        <v>2061</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>2176</v>
+        <v>2158</v>
       </c>
       <c r="D75" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E75" s="0">
-        <v>0.122302293948888</v>
+        <v>0.066879295402785296</v>
       </c>
       <c r="F75" s="0">
-        <v>0.63376068376068395</v>
+        <v>0.48046296296296298</v>
+      </c>
+      <c r="G75" s="0" t="s">
+        <v>2239</v>
       </c>
     </row>
     <row r="76">
@@ -29869,19 +30215,22 @@
         <v>1965</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>2071</v>
+        <v>2062</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>2177</v>
+        <v>2159</v>
       </c>
       <c r="D76" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E76" s="0">
-        <v>0.067405894368252103</v>
+        <v>0.072522522522522504</v>
       </c>
       <c r="F76" s="0">
-        <v>0.57693236714975804</v>
+        <v>0.58412037037037001</v>
+      </c>
+      <c r="G76" s="0" t="s">
+        <v>2240</v>
       </c>
     </row>
     <row r="77">
@@ -29889,19 +30238,22 @@
         <v>1966</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>2072</v>
+        <v>2063</v>
       </c>
       <c r="C77" s="0" t="s">
-        <v>2178</v>
+        <v>2160</v>
       </c>
       <c r="D77" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E77" s="0">
-        <v>0.088422818791946301</v>
+        <v>0.15562080536912801</v>
       </c>
       <c r="F77" s="0">
-        <v>0.59718749999999998</v>
+        <v>0.68346354166666701</v>
+      </c>
+      <c r="G77" s="0" t="s">
+        <v>2241</v>
       </c>
     </row>
     <row r="78">
@@ -29909,19 +30261,22 @@
         <v>1967</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>2073</v>
+        <v>2064</v>
       </c>
       <c r="C78" s="0" t="s">
-        <v>2179</v>
+        <v>2161</v>
       </c>
       <c r="D78" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E78" s="0">
-        <v>0.047717126089068099</v>
+        <v>0.18049500553550499</v>
       </c>
       <c r="F78" s="0">
-        <v>0.50627240143369201</v>
+        <v>0.63445881226053602</v>
+      </c>
+      <c r="G78" s="0" t="s">
+        <v>2242</v>
       </c>
     </row>
     <row r="79">
@@ -29929,19 +30284,22 @@
         <v>1968</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>2074</v>
+        <v>2065</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>2180</v>
+        <v>2162</v>
       </c>
       <c r="D79" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E79" s="0">
-        <v>0.049268018018018001</v>
+        <v>0.0071308724832214801</v>
       </c>
       <c r="F79" s="0">
-        <v>0.60853587962962896</v>
+        <v>0.60026041666666696</v>
+      </c>
+      <c r="G79" s="0" t="s">
+        <v>2243</v>
       </c>
     </row>
     <row r="80">
@@ -29949,19 +30307,22 @@
         <v>1969</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>2075</v>
+        <v>2066</v>
       </c>
       <c r="C80" s="0" t="s">
-        <v>2181</v>
+        <v>2163</v>
       </c>
       <c r="D80" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E80" s="0">
-        <v>0.056385739846252898</v>
+        <v>0.34879929678587401</v>
       </c>
       <c r="F80" s="0">
-        <v>0.66456552706552696</v>
+        <v>0.63118569958847703</v>
+      </c>
+      <c r="G80" s="0" t="s">
+        <v>2244</v>
       </c>
     </row>
     <row r="81">
@@ -29969,19 +30330,22 @@
         <v>1970</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>2076</v>
+        <v>2067</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>2182</v>
+        <v>2164</v>
       </c>
       <c r="D81" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E81" s="0">
-        <v>0.066879295402785296</v>
+        <v>0.0587318087318087</v>
       </c>
       <c r="F81" s="0">
-        <v>0.48046296296296298</v>
+        <v>0.56089743589743602</v>
+      </c>
+      <c r="G81" s="0" t="s">
+        <v>2245</v>
       </c>
     </row>
     <row r="82">
@@ -29989,19 +30353,22 @@
         <v>1971</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>2077</v>
+        <v>2068</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>2183</v>
+        <v>2165</v>
       </c>
       <c r="D82" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E82" s="0">
-        <v>0.072522522522522504</v>
+        <v>0.11755929293242701</v>
       </c>
       <c r="F82" s="0">
-        <v>0.58412037037037001</v>
+        <v>0.73976139601139601</v>
+      </c>
+      <c r="G82" s="0" t="s">
+        <v>2216</v>
       </c>
     </row>
     <row r="83">
@@ -30009,19 +30376,22 @@
         <v>1972</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>2078</v>
+        <v>2069</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>2184</v>
+        <v>2166</v>
       </c>
       <c r="D83" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E83" s="0">
-        <v>0.15562080536912801</v>
+        <v>0.136247657053026</v>
       </c>
       <c r="F83" s="0">
-        <v>0.68346354166666701</v>
+        <v>0.69564814814814802</v>
+      </c>
+      <c r="G83" s="0" t="s">
+        <v>2216</v>
       </c>
     </row>
     <row r="84">
@@ -30029,19 +30399,22 @@
         <v>1973</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>2079</v>
+        <v>2070</v>
       </c>
       <c r="C84" s="0" t="s">
-        <v>2185</v>
+        <v>2167</v>
       </c>
       <c r="D84" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E84" s="0">
-        <v>0.18049500553550499</v>
+        <v>0.11025886864813</v>
       </c>
       <c r="F84" s="0">
-        <v>0.63445881226053602</v>
+        <v>0.59846230158730196</v>
+      </c>
+      <c r="G84" s="0" t="s">
+        <v>2246</v>
       </c>
     </row>
     <row r="85">
@@ -30049,19 +30422,22 @@
         <v>1974</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>2080</v>
+        <v>2071</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>2186</v>
+        <v>2168</v>
       </c>
       <c r="D85" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E85" s="0">
-        <v>0.0071308724832214801</v>
+        <v>0.11696108318753901</v>
       </c>
       <c r="F85" s="0">
-        <v>0.60026041666666696</v>
+        <v>0.67226702508960601</v>
+      </c>
+      <c r="G85" s="0" t="s">
+        <v>2216</v>
       </c>
     </row>
     <row r="86">
@@ -30069,19 +30445,22 @@
         <v>1975</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>2081</v>
+        <v>2072</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>2187</v>
+        <v>2169</v>
       </c>
       <c r="D86" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E86" s="0">
-        <v>0.34879929678587401</v>
+        <v>0</v>
       </c>
       <c r="F86" s="0">
-        <v>0.63118569958847703</v>
+        <v>0.59194444444444405</v>
+      </c>
+      <c r="G86" s="0" t="s">
+        <v>2247</v>
       </c>
     </row>
     <row r="87">
@@ -30089,19 +30468,22 @@
         <v>1976</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>2082</v>
+        <v>2073</v>
       </c>
       <c r="C87" s="0" t="s">
-        <v>2188</v>
+        <v>2170</v>
       </c>
       <c r="D87" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E87" s="0">
-        <v>0.0587318087318087</v>
+        <v>0.058612975391498901</v>
       </c>
       <c r="F87" s="0">
-        <v>0.56089743589743602</v>
+        <v>0.56356481481481502</v>
+      </c>
+      <c r="G87" s="0" t="s">
+        <v>2248</v>
       </c>
     </row>
     <row r="88">
@@ -30109,19 +30491,22 @@
         <v>1977</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>2083</v>
+        <v>2074</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>2189</v>
+        <v>2171</v>
       </c>
       <c r="D88" s="0" t="s">
         <v>1885</v>
       </c>
       <c r="E88" s="0">
-        <v>0.12572706935122999</v>
+        <v>0.072582649763857796</v>
       </c>
       <c r="F88" s="0">
-        <v>0.561574074074074</v>
+        <v>0.52834362139917701</v>
+      </c>
+      <c r="G88" s="0" t="s">
+        <v>2249</v>
       </c>
     </row>
     <row r="89">
@@ -30129,19 +30514,22 @@
         <v>1978</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>2084</v>
+        <v>2075</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>2190</v>
+        <v>2172</v>
       </c>
       <c r="D89" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E89" s="0">
-        <v>0.11755929293242701</v>
+        <v>0.019819819819819801</v>
       </c>
       <c r="F89" s="0">
-        <v>0.73976139601139601</v>
+        <v>0.58087962962963002</v>
+      </c>
+      <c r="G89" s="0" t="s">
+        <v>2235</v>
       </c>
     </row>
     <row r="90">
@@ -30149,19 +30537,22 @@
         <v>1979</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>2085</v>
+        <v>2076</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>2191</v>
+        <v>2173</v>
       </c>
       <c r="D90" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E90" s="0">
-        <v>0.046560402684563802</v>
+        <v>0.098954268768534401</v>
       </c>
       <c r="F90" s="0">
-        <v>0.61927083333333299</v>
+        <v>0.60334302325581402</v>
+      </c>
+      <c r="G90" s="0" t="s">
+        <v>2224</v>
       </c>
     </row>
     <row r="91">
@@ -30169,19 +30560,22 @@
         <v>1980</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>2086</v>
+        <v>2077</v>
       </c>
       <c r="C91" s="0" t="s">
-        <v>2192</v>
+        <v>2174</v>
       </c>
       <c r="D91" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E91" s="0">
-        <v>0.136247657053026</v>
+        <v>0.11534749034749001</v>
       </c>
       <c r="F91" s="0">
-        <v>0.69564814814814802</v>
+        <v>0.422619047619048</v>
+      </c>
+      <c r="G91" s="0" t="s">
+        <v>2212</v>
       </c>
     </row>
     <row r="92">
@@ -30189,19 +30583,22 @@
         <v>1981</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>2087</v>
+        <v>2078</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>2193</v>
+        <v>2175</v>
       </c>
       <c r="D92" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E92" s="0">
-        <v>0.11025886864813</v>
+        <v>0.036912751677852303</v>
       </c>
       <c r="F92" s="0">
-        <v>0.59846230158730196</v>
+        <v>0.56946097883597901</v>
+      </c>
+      <c r="G92" s="0" t="s">
+        <v>2224</v>
       </c>
     </row>
     <row r="93">
@@ -30209,19 +30606,22 @@
         <v>1982</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>2088</v>
+        <v>2079</v>
       </c>
       <c r="C93" s="0" t="s">
-        <v>2194</v>
+        <v>2176</v>
       </c>
       <c r="D93" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E93" s="0">
-        <v>0.11696108318753901</v>
+        <v>0.121621621621622</v>
       </c>
       <c r="F93" s="0">
-        <v>0.67226702508960601</v>
+        <v>0.60429687499999996</v>
+      </c>
+      <c r="G93" s="0" t="s">
+        <v>2220</v>
       </c>
     </row>
     <row r="94">
@@ -30229,19 +30629,22 @@
         <v>1983</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>2089</v>
+        <v>2080</v>
       </c>
       <c r="C94" s="0" t="s">
-        <v>2195</v>
+        <v>2177</v>
       </c>
       <c r="D94" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E94" s="0">
-        <v>0</v>
+        <v>0.024264326277749101</v>
       </c>
       <c r="F94" s="0">
-        <v>0.59194444444444405</v>
+        <v>0.59636752136752103</v>
+      </c>
+      <c r="G94" s="0" t="s">
+        <v>2250</v>
       </c>
     </row>
     <row r="95">
@@ -30249,19 +30652,22 @@
         <v>1984</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>2090</v>
+        <v>2081</v>
       </c>
       <c r="C95" s="0" t="s">
-        <v>2196</v>
+        <v>2178</v>
       </c>
       <c r="D95" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E95" s="0">
-        <v>0.058612975391498901</v>
+        <v>0.45059121621621601</v>
       </c>
       <c r="F95" s="0">
-        <v>0.56356481481481502</v>
+        <v>0.86731770833333299</v>
+      </c>
+      <c r="G95" s="0" t="s">
+        <v>2220</v>
       </c>
     </row>
     <row r="96">
@@ -30269,19 +30675,22 @@
         <v>1985</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>2091</v>
+        <v>2082</v>
       </c>
       <c r="C96" s="0" t="s">
-        <v>2197</v>
+        <v>2179</v>
       </c>
       <c r="D96" s="0" t="s">
-        <v>1885</v>
+        <v>2182</v>
       </c>
       <c r="E96" s="0">
-        <v>0.072582649763857796</v>
+        <v>0.19175455417066201</v>
       </c>
       <c r="F96" s="0">
-        <v>0.52834362139917701</v>
+        <v>0.65466269841269798</v>
+      </c>
+      <c r="G96" s="0" t="s">
+        <v>2203</v>
       </c>
     </row>
     <row r="97">
@@ -30289,19 +30698,22 @@
         <v>1986</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>2092</v>
+        <v>2083</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>2198</v>
+        <v>2180</v>
       </c>
       <c r="D97" s="0" t="s">
-        <v>2210</v>
+        <v>2182</v>
       </c>
       <c r="E97" s="0">
-        <v>0.019819819819819801</v>
+        <v>0.098274209012464003</v>
       </c>
       <c r="F97" s="0">
-        <v>0.58087962962963002</v>
+        <v>0.60391865079365104</v>
+      </c>
+      <c r="G97" s="0" t="s">
+        <v>2196</v>
       </c>
     </row>
     <row r="98">
@@ -30309,199 +30721,22 @@
         <v>1987</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>2093</v>
+        <v>2084</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>2199</v>
+        <v>2181</v>
       </c>
       <c r="D98" s="0" t="s">
-        <v>2210</v>
+        <v>2182</v>
       </c>
       <c r="E98" s="0">
-        <v>0.098954268768534401</v>
+        <v>0.105855855855856</v>
       </c>
       <c r="F98" s="0">
-        <v>0.60334302325581402</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="0" t="s">
-        <v>1988</v>
-      </c>
-      <c r="B99" s="0" t="s">
-        <v>2094</v>
-      </c>
-      <c r="C99" s="0" t="s">
-        <v>2200</v>
-      </c>
-      <c r="D99" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E99" s="0">
-        <v>0.11534749034749001</v>
-      </c>
-      <c r="F99" s="0">
-        <v>0.422619047619048</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="0" t="s">
-        <v>1989</v>
-      </c>
-      <c r="B100" s="0" t="s">
-        <v>2095</v>
-      </c>
-      <c r="C100" s="0" t="s">
-        <v>2201</v>
-      </c>
-      <c r="D100" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E100" s="0">
-        <v>0.036912751677852303</v>
-      </c>
-      <c r="F100" s="0">
-        <v>0.56946097883597901</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="0" t="s">
-        <v>1990</v>
-      </c>
-      <c r="B101" s="0" t="s">
-        <v>2096</v>
-      </c>
-      <c r="C101" s="0" t="s">
-        <v>2202</v>
-      </c>
-      <c r="D101" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E101" s="0">
-        <v>0.121621621621622</v>
-      </c>
-      <c r="F101" s="0">
-        <v>0.60429687499999996</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="0" t="s">
-        <v>1991</v>
-      </c>
-      <c r="B102" s="0" t="s">
-        <v>2097</v>
-      </c>
-      <c r="C102" s="0" t="s">
-        <v>2203</v>
-      </c>
-      <c r="D102" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E102" s="0">
-        <v>0.024264326277749101</v>
-      </c>
-      <c r="F102" s="0">
-        <v>0.59636752136752103</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="0" t="s">
-        <v>1992</v>
-      </c>
-      <c r="B103" s="0" t="s">
-        <v>2098</v>
-      </c>
-      <c r="C103" s="0" t="s">
-        <v>2204</v>
-      </c>
-      <c r="D103" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E103" s="0">
-        <v>0.45059121621621601</v>
-      </c>
-      <c r="F103" s="0">
-        <v>0.86731770833333299</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="0" t="s">
-        <v>1993</v>
-      </c>
-      <c r="B104" s="0" t="s">
-        <v>2099</v>
-      </c>
-      <c r="C104" s="0" t="s">
-        <v>2205</v>
-      </c>
-      <c r="D104" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E104" s="0">
-        <v>0.19175455417066201</v>
-      </c>
-      <c r="F104" s="0">
-        <v>0.65466269841269798</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="0" t="s">
-        <v>1994</v>
-      </c>
-      <c r="B105" s="0" t="s">
-        <v>2100</v>
-      </c>
-      <c r="C105" s="0" t="s">
-        <v>2206</v>
-      </c>
-      <c r="D105" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E105" s="0">
-        <v>0.098274209012464003</v>
-      </c>
-      <c r="F105" s="0">
-        <v>0.60391865079365104</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="0" t="s">
-        <v>1995</v>
-      </c>
-      <c r="B106" s="0" t="s">
-        <v>2101</v>
-      </c>
-      <c r="C106" s="0" t="s">
-        <v>2207</v>
-      </c>
-      <c r="D106" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E106" s="0">
-        <v>0.121700223713647</v>
-      </c>
-      <c r="F106" s="0">
-        <v>0.63953703703703702</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="0" t="s">
-        <v>1996</v>
-      </c>
-      <c r="B107" s="0" t="s">
-        <v>2102</v>
-      </c>
-      <c r="C107" s="0" t="s">
-        <v>2208</v>
-      </c>
-      <c r="D107" s="0" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E107" s="0">
-        <v>0.105855855855856</v>
-      </c>
-      <c r="F107" s="0">
         <v>0.60138888888888897</v>
+      </c>
+      <c r="G98" s="0" t="s">
+        <v>2186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>